<commit_message>
feat: Modulnummer-Spalte für Zusatzmodule (wird Modul-ID)
Neue Spalte 'Modulnummer' in der Excel-Vorlage; der Konverter mappt sie
auf planSemesterModulId, das im Dashboard als Modul-ID dient und das
auto-generierte EXTRA_<n> ersetzt. Leer lassen -> weiterhin Fallback-ID.
.gitignore: Excel-Lock-Dateien (~$*.xlsx) ausschliessen.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/Vorlage_Zusatzmodule.xlsx
+++ b/tools/Vorlage_Zusatzmodule.xlsx
@@ -251,87 +251,87 @@
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>Optional. Englischer Titel.</t>
+        <t>Empfohlen. Eindeutige Modulnummer/-kennung; wird im Dashboard als Modul-ID verwendet. Leer lassen -&gt; automatische ID.</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>Deutsch / Englisch / Bilingual.</t>
+        <t>Optional. Englischer Titel.</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
-        <t>Name(n) der Dozierenden. Mehrere mit Komma trennen.</t>
+        <t>Deutsch / Englisch / Bilingual.</t>
       </text>
     </comment>
     <comment ref="H1" authorId="0" shapeId="0">
       <text>
-        <t>Optional. Modulverantwortliche Person.</t>
+        <t>Name(n) der Dozierenden. Mehrere mit Komma trennen.</t>
       </text>
     </comment>
     <comment ref="I1" authorId="0" shapeId="0">
       <text>
-        <t>Optional. Durchführungsort.</t>
+        <t>Optional. Modulverantwortliche Person.</t>
       </text>
     </comment>
     <comment ref="J1" authorId="0" shapeId="0">
       <text>
-        <t>Optional, z.B. Pflicht- / Wahlmodul.</t>
+        <t>Optional. Durchführungsort.</t>
       </text>
     </comment>
     <comment ref="K1" authorId="0" shapeId="0">
       <text>
-        <t>Fliesstext. Beschreibung des Inhalts.</t>
+        <t>Optional, z.B. Pflicht- / Wahlmodul.</t>
       </text>
     </comment>
     <comment ref="L1" authorId="0" shapeId="0">
       <text>
-        <t>Optional. Kernidee / Leitgedanke.</t>
+        <t>Fliesstext. Beschreibung des Inhalts.</t>
       </text>
     </comment>
     <comment ref="M1" authorId="0" shapeId="0">
       <text>
-        <t>Optional. Erworbene Kompetenzen.</t>
+        <t>Optional. Kernidee / Leitgedanke.</t>
       </text>
     </comment>
     <comment ref="N1" authorId="0" shapeId="0">
       <text>
-        <t>Optional. Literaturangaben.</t>
+        <t>Optional. Erworbene Kompetenzen.</t>
       </text>
     </comment>
     <comment ref="O1" authorId="0" shapeId="0">
       <text>
-        <t>Optional. Voraussetzungen.</t>
+        <t>Optional. Literaturangaben.</t>
       </text>
     </comment>
     <comment ref="P1" authorId="0" shapeId="0">
       <text>
-        <t>Optional. Art des Leistungsnachweises.</t>
+        <t>Optional. Voraussetzungen.</t>
       </text>
     </comment>
     <comment ref="Q1" authorId="0" shapeId="0">
       <text>
-        <t>Optional. Link zur Modulbeschreibung.</t>
+        <t>Optional. Art des Leistungsnachweises.</t>
       </text>
     </comment>
     <comment ref="R1" authorId="0" shapeId="0">
       <text>
-        <t>Optional (Stundenplan). Wochentag aus der Auswahlliste.</t>
+        <t>Optional. Link zur Modulbeschreibung.</t>
       </text>
     </comment>
     <comment ref="S1" authorId="0" shapeId="0">
       <text>
-        <t>Optional (Stundenplan). Format HH:MM, z.B. 10:15.</t>
+        <t>Optional (Stundenplan). Wochentag aus der Auswahlliste.</t>
       </text>
     </comment>
     <comment ref="T1" authorId="0" shapeId="0">
       <text>
-        <t>Optional (Stundenplan). Format HH:MM, z.B. 12:00.</t>
+        <t>Optional (Stundenplan). Format HH:MM, z.B. 10:15.</t>
       </text>
     </comment>
     <comment ref="U1" authorId="0" shapeId="0">
       <text>
-        <t>Optional (Stundenplan). Format TT.MM.JJJJ.</t>
+        <t>Optional (Stundenplan). Format HH:MM, z.B. 12:00.</t>
       </text>
     </comment>
     <comment ref="V1" authorId="0" shapeId="0">
@@ -341,10 +341,15 @@
     </comment>
     <comment ref="W1" authorId="0" shapeId="0">
       <text>
+        <t>Optional (Stundenplan). Format TT.MM.JJJJ.</t>
+      </text>
+    </comment>
+    <comment ref="X1" authorId="0" shapeId="0">
+      <text>
         <t>Optional (Stundenplan). Alle Daten TT.MM.JJJJ, mit Semikolon (;) getrennt.</t>
       </text>
     </comment>
-    <comment ref="X1" authorId="0" shapeId="0">
+    <comment ref="Y1" authorId="0" shapeId="0">
       <text>
         <t>Optional (Stundenplan). Raum(e). Mehrere mit Komma trennen.</t>
       </text>
@@ -647,7 +652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -790,7 +795,7 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>Modultitel (Englisch)</t>
+          <t>Modulnummer</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
@@ -800,19 +805,19 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Optional. Englischer Titel.</t>
+          <t>Empfohlen. Eindeutige Modulnummer/-kennung; wird im Dashboard als Modul-ID verwendet. Leer lassen -&gt; automatische ID.</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>z.B. Test Module A (external)</t>
+          <t>z.B. EXT-INF-101</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>Unterrichtssprache</t>
+          <t>Modultitel (Englisch)</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
@@ -822,19 +827,19 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Deutsch / Englisch / Bilingual.</t>
+          <t>Optional. Englischer Titel.</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>z.B. Deutsch</t>
+          <t>z.B. Test Module A (external)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>Dozierende</t>
+          <t>Unterrichtssprache</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
@@ -844,19 +849,19 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Name(n) der Dozierenden. Mehrere mit Komma trennen.</t>
+          <t>Deutsch / Englisch / Bilingual.</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>z.B. Vorname Nachname</t>
+          <t>z.B. Deutsch</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>Modulverantwortung</t>
+          <t>Dozierende</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
@@ -866,7 +871,7 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Optional. Modulverantwortliche Person.</t>
+          <t>Name(n) der Dozierenden. Mehrere mit Komma trennen.</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
@@ -878,7 +883,7 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Standort / Ort</t>
+          <t>Modulverantwortung</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
@@ -888,19 +893,19 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Optional. Durchführungsort.</t>
+          <t>Optional. Modulverantwortliche Person.</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>z.B. Olten</t>
+          <t>z.B. Vorname Nachname</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>Modultyp</t>
+          <t>Standort / Ort</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
@@ -910,19 +915,19 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Optional, z.B. Pflicht- / Wahlmodul.</t>
+          <t>Optional. Durchführungsort.</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>z.B. Wahlmodul</t>
+          <t>z.B. Olten</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>Modulinhalt / Beschreibung</t>
+          <t>Modultyp</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
@@ -932,19 +937,19 @@
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Fliesstext. Beschreibung des Inhalts.</t>
+          <t>Optional, z.B. Pflicht- / Wahlmodul.</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>z.B. Kurzbeschreibung des Modulinhalts …</t>
+          <t>z.B. Wahlmodul</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>Kernidee</t>
+          <t>Modulinhalt / Beschreibung</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
@@ -954,15 +959,19 @@
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Optional. Kernidee / Leitgedanke.</t>
-        </is>
-      </c>
-      <c r="D18" s="8" t="inlineStr"/>
+          <t>Fliesstext. Beschreibung des Inhalts.</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>z.B. Kurzbeschreibung des Modulinhalts …</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>Kompetenzen</t>
+          <t>Kernidee</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
@@ -972,19 +981,15 @@
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Optional. Erworbene Kompetenzen.</t>
-        </is>
-      </c>
-      <c r="D19" s="8" t="inlineStr">
-        <is>
-          <t>z.B. Beispielkompetenz 1, Beispielkompetenz 2</t>
-        </is>
-      </c>
+          <t>Optional. Kernidee / Leitgedanke.</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>Literatur</t>
+          <t>Kompetenzen</t>
         </is>
       </c>
       <c r="B20" s="8" t="inlineStr">
@@ -994,15 +999,19 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Optional. Literaturangaben.</t>
-        </is>
-      </c>
-      <c r="D20" s="8" t="inlineStr"/>
+          <t>Optional. Erworbene Kompetenzen.</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>z.B. Beispielkompetenz 1, Beispielkompetenz 2</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>Voraussetzungen</t>
+          <t>Literatur</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
@@ -1012,19 +1021,15 @@
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Optional. Voraussetzungen.</t>
-        </is>
-      </c>
-      <c r="D21" s="8" t="inlineStr">
-        <is>
-          <t>z.B. Keine besonderen Voraussetzungen.</t>
-        </is>
-      </c>
+          <t>Optional. Literaturangaben.</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>Leistungsnachweis</t>
+          <t>Voraussetzungen</t>
         </is>
       </c>
       <c r="B22" s="8" t="inlineStr">
@@ -1034,19 +1039,19 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Optional. Art des Leistungsnachweises.</t>
+          <t>Optional. Voraussetzungen.</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>z.B. Schriftliche Prüfung</t>
+          <t>z.B. Keine besonderen Voraussetzungen.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>Link (URL)</t>
+          <t>Leistungsnachweis</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
@@ -1056,19 +1061,19 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Optional. Link zur Modulbeschreibung.</t>
+          <t>Optional. Art des Leistungsnachweises.</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>z.B. https://www.fhnw.ch</t>
+          <t>z.B. Schriftliche Prüfung</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>Wochentag</t>
+          <t>Link (URL)</t>
         </is>
       </c>
       <c r="B24" s="8" t="inlineStr">
@@ -1078,19 +1083,19 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Optional (Stundenplan). Wochentag aus der Auswahlliste.</t>
+          <t>Optional. Link zur Modulbeschreibung.</t>
         </is>
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
-          <t>z.B. Montag</t>
+          <t>z.B. https://www.fhnw.ch</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>Zeit von</t>
+          <t>Wochentag</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
@@ -1100,19 +1105,19 @@
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Optional (Stundenplan). Format HH:MM, z.B. 10:15.</t>
+          <t>Optional (Stundenplan). Wochentag aus der Auswahlliste.</t>
         </is>
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>z.B. 10:15</t>
+          <t>z.B. Montag</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>Zeit bis</t>
+          <t>Zeit von</t>
         </is>
       </c>
       <c r="B26" s="8" t="inlineStr">
@@ -1122,19 +1127,19 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Optional (Stundenplan). Format HH:MM, z.B. 12:00.</t>
+          <t>Optional (Stundenplan). Format HH:MM, z.B. 10:15.</t>
         </is>
       </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>z.B. 12:00</t>
+          <t>z.B. 10:15</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>Erster Termin</t>
+          <t>Zeit bis</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
@@ -1144,19 +1149,19 @@
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Optional (Stundenplan). Format TT.MM.JJJJ.</t>
+          <t>Optional (Stundenplan). Format HH:MM, z.B. 12:00.</t>
         </is>
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>z.B. 14.09.2026</t>
+          <t>z.B. 12:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>Letzter Termin</t>
+          <t>Erster Termin</t>
         </is>
       </c>
       <c r="B28" s="8" t="inlineStr">
@@ -1171,14 +1176,14 @@
       </c>
       <c r="D28" s="8" t="inlineStr">
         <is>
-          <t>z.B. 21.12.2026</t>
+          <t>z.B. 14.09.2026</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>Alle Termine</t>
+          <t>Letzter Termin</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
@@ -1188,44 +1193,66 @@
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Optional (Stundenplan). Alle Daten TT.MM.JJJJ, mit Semikolon (;) getrennt.</t>
+          <t>Optional (Stundenplan). Format TT.MM.JJJJ.</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>z.B. 14.09.2026; 21.09.2026; 28.09.2026</t>
+          <t>z.B. 21.12.2026</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
+          <t>Alle Termine</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Optional (Stundenplan). Alle Daten TT.MM.JJJJ, mit Semikolon (;) getrennt.</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>z.B. 14.09.2026; 21.09.2026; 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
           <t>Raum / Räume</t>
         </is>
       </c>
-      <c r="B30" s="8" t="inlineStr">
+      <c r="B31" s="8" t="inlineStr">
         <is>
           <t>optional</t>
         </is>
       </c>
-      <c r="C30" s="7" t="inlineStr">
+      <c r="C31" s="7" t="inlineStr">
         <is>
           <t>Optional (Stundenplan). Raum(e). Mehrere mit Komma trennen.</t>
         </is>
       </c>
-      <c r="D30" s="8" t="inlineStr">
+      <c r="D31" s="8" t="inlineStr">
         <is>
           <t>z.B. Beispielraum 1.234</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="9" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="9" t="inlineStr">
         <is>
           <t>Zurückgeben an:</t>
         </is>
       </c>
-      <c r="C32" s="10" t="inlineStr">
+      <c r="C33" s="10" t="inlineStr">
         <is>
           <t>die für den Modulplaner verantwortliche Person (ausgefülltes Excel).</t>
         </is>
@@ -1246,33 +1273,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X59"/>
+  <dimension ref="A1:Y59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="40" customWidth="1" min="11" max="11"/>
-    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
     <col width="30" customWidth="1" min="13" max="13"/>
-    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="30" customWidth="1" min="14" max="14"/>
     <col width="24" customWidth="1" min="15" max="15"/>
-    <col width="22" customWidth="1" min="16" max="16"/>
-    <col width="28" customWidth="1" min="17" max="17"/>
-    <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="24" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
+    <col width="28" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
     <col width="10" customWidth="1" min="20" max="20"/>
-    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
     <col width="14" customWidth="1" min="22" max="22"/>
-    <col width="40" customWidth="1" min="23" max="23"/>
-    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="40" customWidth="1" min="24" max="24"/>
+    <col width="18" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -1298,100 +1326,105 @@
       </c>
       <c r="E1" s="12" t="inlineStr">
         <is>
+          <t>Modulnummer</t>
+        </is>
+      </c>
+      <c r="F1" s="12" t="inlineStr">
+        <is>
           <t>Modultitel (Englisch)</t>
         </is>
       </c>
-      <c r="F1" s="12" t="inlineStr">
+      <c r="G1" s="12" t="inlineStr">
         <is>
           <t>Unterrichtssprache</t>
         </is>
       </c>
-      <c r="G1" s="12" t="inlineStr">
+      <c r="H1" s="12" t="inlineStr">
         <is>
           <t>Dozierende</t>
         </is>
       </c>
-      <c r="H1" s="12" t="inlineStr">
+      <c r="I1" s="12" t="inlineStr">
         <is>
           <t>Modulverantwortung</t>
         </is>
       </c>
-      <c r="I1" s="12" t="inlineStr">
+      <c r="J1" s="12" t="inlineStr">
         <is>
           <t>Standort / Ort</t>
         </is>
       </c>
-      <c r="J1" s="12" t="inlineStr">
+      <c r="K1" s="12" t="inlineStr">
         <is>
           <t>Modultyp</t>
         </is>
       </c>
-      <c r="K1" s="12" t="inlineStr">
+      <c r="L1" s="12" t="inlineStr">
         <is>
           <t>Modulinhalt / Beschreibung</t>
         </is>
       </c>
-      <c r="L1" s="12" t="inlineStr">
+      <c r="M1" s="12" t="inlineStr">
         <is>
           <t>Kernidee</t>
         </is>
       </c>
-      <c r="M1" s="12" t="inlineStr">
+      <c r="N1" s="12" t="inlineStr">
         <is>
           <t>Kompetenzen</t>
         </is>
       </c>
-      <c r="N1" s="12" t="inlineStr">
+      <c r="O1" s="12" t="inlineStr">
         <is>
           <t>Literatur</t>
         </is>
       </c>
-      <c r="O1" s="12" t="inlineStr">
+      <c r="P1" s="12" t="inlineStr">
         <is>
           <t>Voraussetzungen</t>
         </is>
       </c>
-      <c r="P1" s="12" t="inlineStr">
+      <c r="Q1" s="12" t="inlineStr">
         <is>
           <t>Leistungsnachweis</t>
         </is>
       </c>
-      <c r="Q1" s="12" t="inlineStr">
+      <c r="R1" s="12" t="inlineStr">
         <is>
           <t>Link (URL)</t>
         </is>
       </c>
-      <c r="R1" s="12" t="inlineStr">
+      <c r="S1" s="12" t="inlineStr">
         <is>
           <t>Wochentag</t>
         </is>
       </c>
-      <c r="S1" s="12" t="inlineStr">
+      <c r="T1" s="12" t="inlineStr">
         <is>
           <t>Zeit von</t>
         </is>
       </c>
-      <c r="T1" s="12" t="inlineStr">
+      <c r="U1" s="12" t="inlineStr">
         <is>
           <t>Zeit bis</t>
         </is>
       </c>
-      <c r="U1" s="12" t="inlineStr">
+      <c r="V1" s="12" t="inlineStr">
         <is>
           <t>Erster Termin</t>
         </is>
       </c>
-      <c r="V1" s="12" t="inlineStr">
+      <c r="W1" s="12" t="inlineStr">
         <is>
           <t>Letzter Termin</t>
         </is>
       </c>
-      <c r="W1" s="12" t="inlineStr">
+      <c r="X1" s="12" t="inlineStr">
         <is>
           <t>Alle Termine</t>
         </is>
       </c>
-      <c r="X1" s="12" t="inlineStr">
+      <c r="Y1" s="12" t="inlineStr">
         <is>
           <t>Raum / Räume</t>
         </is>
@@ -1418,92 +1451,97 @@
       </c>
       <c r="E2" s="13" t="inlineStr">
         <is>
+          <t>EXT-INF-101</t>
+        </is>
+      </c>
+      <c r="F2" s="13" t="inlineStr">
+        <is>
           <t>Test Module A (external)</t>
         </is>
       </c>
-      <c r="F2" s="13" t="inlineStr">
+      <c r="G2" s="13" t="inlineStr">
         <is>
           <t>Deutsch</t>
         </is>
       </c>
-      <c r="G2" s="13" t="inlineStr">
+      <c r="H2" s="13" t="inlineStr">
         <is>
           <t>Vorname Nachname</t>
         </is>
       </c>
-      <c r="H2" s="13" t="inlineStr">
+      <c r="I2" s="13" t="inlineStr">
         <is>
           <t>Vorname Nachname</t>
         </is>
       </c>
-      <c r="I2" s="13" t="inlineStr">
+      <c r="J2" s="13" t="inlineStr">
         <is>
           <t>Olten</t>
         </is>
       </c>
-      <c r="J2" s="13" t="inlineStr">
+      <c r="K2" s="13" t="inlineStr">
         <is>
           <t>Wahlmodul</t>
         </is>
       </c>
-      <c r="K2" s="13" t="inlineStr">
+      <c r="L2" s="13" t="inlineStr">
         <is>
           <t>Kurzbeschreibung des Modulinhalts …</t>
         </is>
       </c>
-      <c r="L2" s="13" t="n"/>
-      <c r="M2" s="13" t="inlineStr">
+      <c r="M2" s="13" t="n"/>
+      <c r="N2" s="13" t="inlineStr">
         <is>
           <t>Beispielkompetenz 1, Beispielkompetenz 2</t>
         </is>
       </c>
-      <c r="N2" s="13" t="n"/>
-      <c r="O2" s="13" t="inlineStr">
+      <c r="O2" s="13" t="n"/>
+      <c r="P2" s="13" t="inlineStr">
         <is>
           <t>Keine besonderen Voraussetzungen.</t>
         </is>
       </c>
-      <c r="P2" s="13" t="inlineStr">
+      <c r="Q2" s="13" t="inlineStr">
         <is>
           <t>Schriftliche Prüfung</t>
         </is>
       </c>
-      <c r="Q2" s="13" t="inlineStr">
+      <c r="R2" s="13" t="inlineStr">
         <is>
           <t>https://www.fhnw.ch</t>
         </is>
       </c>
-      <c r="R2" s="13" t="inlineStr">
+      <c r="S2" s="13" t="inlineStr">
         <is>
           <t>Montag</t>
         </is>
       </c>
-      <c r="S2" s="13" t="inlineStr">
+      <c r="T2" s="13" t="inlineStr">
         <is>
           <t>10:15</t>
         </is>
       </c>
-      <c r="T2" s="13" t="inlineStr">
+      <c r="U2" s="13" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="U2" s="13" t="inlineStr">
+      <c r="V2" s="13" t="inlineStr">
         <is>
           <t>14.09.2026</t>
         </is>
       </c>
-      <c r="V2" s="13" t="inlineStr">
+      <c r="W2" s="13" t="inlineStr">
         <is>
           <t>21.12.2026</t>
         </is>
       </c>
-      <c r="W2" s="13" t="inlineStr">
+      <c r="X2" s="13" t="inlineStr">
         <is>
           <t>14.09.2026; 21.09.2026; 28.09.2026</t>
         </is>
       </c>
-      <c r="X2" s="13" t="inlineStr">
+      <c r="Y2" s="13" t="inlineStr">
         <is>
           <t>Beispielraum 1.234</t>
         </is>
@@ -1530,60 +1568,65 @@
       </c>
       <c r="E3" s="13" t="inlineStr">
         <is>
+          <t>EXT-INF-102</t>
+        </is>
+      </c>
+      <c r="F3" s="13" t="inlineStr">
+        <is>
           <t>Test Module B (external)</t>
         </is>
       </c>
-      <c r="F3" s="13" t="inlineStr">
+      <c r="G3" s="13" t="inlineStr">
         <is>
           <t>Deutsch</t>
         </is>
       </c>
-      <c r="G3" s="13" t="inlineStr">
+      <c r="H3" s="13" t="inlineStr">
         <is>
           <t>Andere Person</t>
         </is>
       </c>
-      <c r="H3" s="13" t="inlineStr">
+      <c r="I3" s="13" t="inlineStr">
         <is>
           <t>Andere Person</t>
         </is>
       </c>
-      <c r="I3" s="13" t="inlineStr">
+      <c r="J3" s="13" t="inlineStr">
         <is>
           <t>Brugg-Windisch</t>
         </is>
       </c>
-      <c r="J3" s="13" t="inlineStr">
+      <c r="K3" s="13" t="inlineStr">
         <is>
           <t>Pflichtmodul</t>
         </is>
       </c>
-      <c r="K3" s="13" t="inlineStr">
+      <c r="L3" s="13" t="inlineStr">
         <is>
           <t>Kurzbeschreibung des Modulinhalts …</t>
         </is>
       </c>
-      <c r="L3" s="13" t="n"/>
       <c r="M3" s="13" t="n"/>
       <c r="N3" s="13" t="n"/>
       <c r="O3" s="13" t="n"/>
-      <c r="P3" s="13" t="inlineStr">
+      <c r="P3" s="13" t="n"/>
+      <c r="Q3" s="13" t="inlineStr">
         <is>
           <t>Projektarbeit</t>
         </is>
       </c>
-      <c r="Q3" s="13" t="inlineStr">
+      <c r="R3" s="13" t="inlineStr">
         <is>
           <t>https://www.fhnw.ch</t>
         </is>
       </c>
-      <c r="R3" s="13" t="n"/>
       <c r="S3" s="13" t="n"/>
       <c r="T3" s="13" t="n"/>
       <c r="U3" s="13" t="n"/>
       <c r="V3" s="13" t="n"/>
       <c r="W3" s="13" t="n"/>
       <c r="X3" s="13" t="n"/>
+      <c r="Y3" s="13" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n"/>
@@ -1610,6 +1653,7 @@
       <c r="V4" s="7" t="n"/>
       <c r="W4" s="7" t="n"/>
       <c r="X4" s="7" t="n"/>
+      <c r="Y4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n"/>
@@ -1636,6 +1680,7 @@
       <c r="V5" s="7" t="n"/>
       <c r="W5" s="7" t="n"/>
       <c r="X5" s="7" t="n"/>
+      <c r="Y5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n"/>
@@ -1662,6 +1707,7 @@
       <c r="V6" s="7" t="n"/>
       <c r="W6" s="7" t="n"/>
       <c r="X6" s="7" t="n"/>
+      <c r="Y6" s="7" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n"/>
@@ -1688,6 +1734,7 @@
       <c r="V7" s="7" t="n"/>
       <c r="W7" s="7" t="n"/>
       <c r="X7" s="7" t="n"/>
+      <c r="Y7" s="7" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n"/>
@@ -1714,6 +1761,7 @@
       <c r="V8" s="7" t="n"/>
       <c r="W8" s="7" t="n"/>
       <c r="X8" s="7" t="n"/>
+      <c r="Y8" s="7" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n"/>
@@ -1740,6 +1788,7 @@
       <c r="V9" s="7" t="n"/>
       <c r="W9" s="7" t="n"/>
       <c r="X9" s="7" t="n"/>
+      <c r="Y9" s="7" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n"/>
@@ -1766,6 +1815,7 @@
       <c r="V10" s="7" t="n"/>
       <c r="W10" s="7" t="n"/>
       <c r="X10" s="7" t="n"/>
+      <c r="Y10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n"/>
@@ -1792,6 +1842,7 @@
       <c r="V11" s="7" t="n"/>
       <c r="W11" s="7" t="n"/>
       <c r="X11" s="7" t="n"/>
+      <c r="Y11" s="7" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n"/>
@@ -1818,6 +1869,7 @@
       <c r="V12" s="7" t="n"/>
       <c r="W12" s="7" t="n"/>
       <c r="X12" s="7" t="n"/>
+      <c r="Y12" s="7" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n"/>
@@ -1844,6 +1896,7 @@
       <c r="V13" s="7" t="n"/>
       <c r="W13" s="7" t="n"/>
       <c r="X13" s="7" t="n"/>
+      <c r="Y13" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n"/>
@@ -1870,6 +1923,7 @@
       <c r="V14" s="7" t="n"/>
       <c r="W14" s="7" t="n"/>
       <c r="X14" s="7" t="n"/>
+      <c r="Y14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n"/>
@@ -1896,6 +1950,7 @@
       <c r="V15" s="7" t="n"/>
       <c r="W15" s="7" t="n"/>
       <c r="X15" s="7" t="n"/>
+      <c r="Y15" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n"/>
@@ -1922,6 +1977,7 @@
       <c r="V16" s="7" t="n"/>
       <c r="W16" s="7" t="n"/>
       <c r="X16" s="7" t="n"/>
+      <c r="Y16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n"/>
@@ -1948,6 +2004,7 @@
       <c r="V17" s="7" t="n"/>
       <c r="W17" s="7" t="n"/>
       <c r="X17" s="7" t="n"/>
+      <c r="Y17" s="7" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n"/>
@@ -1974,6 +2031,7 @@
       <c r="V18" s="7" t="n"/>
       <c r="W18" s="7" t="n"/>
       <c r="X18" s="7" t="n"/>
+      <c r="Y18" s="7" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n"/>
@@ -2000,6 +2058,7 @@
       <c r="V19" s="7" t="n"/>
       <c r="W19" s="7" t="n"/>
       <c r="X19" s="7" t="n"/>
+      <c r="Y19" s="7" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="n"/>
@@ -2026,6 +2085,7 @@
       <c r="V20" s="7" t="n"/>
       <c r="W20" s="7" t="n"/>
       <c r="X20" s="7" t="n"/>
+      <c r="Y20" s="7" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="n"/>
@@ -2052,6 +2112,7 @@
       <c r="V21" s="7" t="n"/>
       <c r="W21" s="7" t="n"/>
       <c r="X21" s="7" t="n"/>
+      <c r="Y21" s="7" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="n"/>
@@ -2078,6 +2139,7 @@
       <c r="V22" s="7" t="n"/>
       <c r="W22" s="7" t="n"/>
       <c r="X22" s="7" t="n"/>
+      <c r="Y22" s="7" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="n"/>
@@ -2104,6 +2166,7 @@
       <c r="V23" s="7" t="n"/>
       <c r="W23" s="7" t="n"/>
       <c r="X23" s="7" t="n"/>
+      <c r="Y23" s="7" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n"/>
@@ -2130,6 +2193,7 @@
       <c r="V24" s="7" t="n"/>
       <c r="W24" s="7" t="n"/>
       <c r="X24" s="7" t="n"/>
+      <c r="Y24" s="7" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n"/>
@@ -2156,6 +2220,7 @@
       <c r="V25" s="7" t="n"/>
       <c r="W25" s="7" t="n"/>
       <c r="X25" s="7" t="n"/>
+      <c r="Y25" s="7" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="n"/>
@@ -2182,6 +2247,7 @@
       <c r="V26" s="7" t="n"/>
       <c r="W26" s="7" t="n"/>
       <c r="X26" s="7" t="n"/>
+      <c r="Y26" s="7" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="n"/>
@@ -2208,6 +2274,7 @@
       <c r="V27" s="7" t="n"/>
       <c r="W27" s="7" t="n"/>
       <c r="X27" s="7" t="n"/>
+      <c r="Y27" s="7" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="n"/>
@@ -2234,6 +2301,7 @@
       <c r="V28" s="7" t="n"/>
       <c r="W28" s="7" t="n"/>
       <c r="X28" s="7" t="n"/>
+      <c r="Y28" s="7" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="n"/>
@@ -2260,6 +2328,7 @@
       <c r="V29" s="7" t="n"/>
       <c r="W29" s="7" t="n"/>
       <c r="X29" s="7" t="n"/>
+      <c r="Y29" s="7" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="n"/>
@@ -2286,6 +2355,7 @@
       <c r="V30" s="7" t="n"/>
       <c r="W30" s="7" t="n"/>
       <c r="X30" s="7" t="n"/>
+      <c r="Y30" s="7" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="n"/>
@@ -2312,6 +2382,7 @@
       <c r="V31" s="7" t="n"/>
       <c r="W31" s="7" t="n"/>
       <c r="X31" s="7" t="n"/>
+      <c r="Y31" s="7" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="n"/>
@@ -2338,6 +2409,7 @@
       <c r="V32" s="7" t="n"/>
       <c r="W32" s="7" t="n"/>
       <c r="X32" s="7" t="n"/>
+      <c r="Y32" s="7" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="n"/>
@@ -2364,6 +2436,7 @@
       <c r="V33" s="7" t="n"/>
       <c r="W33" s="7" t="n"/>
       <c r="X33" s="7" t="n"/>
+      <c r="Y33" s="7" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="n"/>
@@ -2390,6 +2463,7 @@
       <c r="V34" s="7" t="n"/>
       <c r="W34" s="7" t="n"/>
       <c r="X34" s="7" t="n"/>
+      <c r="Y34" s="7" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="n"/>
@@ -2416,6 +2490,7 @@
       <c r="V35" s="7" t="n"/>
       <c r="W35" s="7" t="n"/>
       <c r="X35" s="7" t="n"/>
+      <c r="Y35" s="7" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="n"/>
@@ -2442,6 +2517,7 @@
       <c r="V36" s="7" t="n"/>
       <c r="W36" s="7" t="n"/>
       <c r="X36" s="7" t="n"/>
+      <c r="Y36" s="7" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="n"/>
@@ -2468,6 +2544,7 @@
       <c r="V37" s="7" t="n"/>
       <c r="W37" s="7" t="n"/>
       <c r="X37" s="7" t="n"/>
+      <c r="Y37" s="7" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="n"/>
@@ -2494,6 +2571,7 @@
       <c r="V38" s="7" t="n"/>
       <c r="W38" s="7" t="n"/>
       <c r="X38" s="7" t="n"/>
+      <c r="Y38" s="7" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="n"/>
@@ -2520,6 +2598,7 @@
       <c r="V39" s="7" t="n"/>
       <c r="W39" s="7" t="n"/>
       <c r="X39" s="7" t="n"/>
+      <c r="Y39" s="7" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="n"/>
@@ -2546,6 +2625,7 @@
       <c r="V40" s="7" t="n"/>
       <c r="W40" s="7" t="n"/>
       <c r="X40" s="7" t="n"/>
+      <c r="Y40" s="7" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="n"/>
@@ -2572,6 +2652,7 @@
       <c r="V41" s="7" t="n"/>
       <c r="W41" s="7" t="n"/>
       <c r="X41" s="7" t="n"/>
+      <c r="Y41" s="7" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="n"/>
@@ -2598,6 +2679,7 @@
       <c r="V42" s="7" t="n"/>
       <c r="W42" s="7" t="n"/>
       <c r="X42" s="7" t="n"/>
+      <c r="Y42" s="7" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="n"/>
@@ -2624,6 +2706,7 @@
       <c r="V43" s="7" t="n"/>
       <c r="W43" s="7" t="n"/>
       <c r="X43" s="7" t="n"/>
+      <c r="Y43" s="7" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="n"/>
@@ -2650,6 +2733,7 @@
       <c r="V44" s="7" t="n"/>
       <c r="W44" s="7" t="n"/>
       <c r="X44" s="7" t="n"/>
+      <c r="Y44" s="7" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="n"/>
@@ -2676,6 +2760,7 @@
       <c r="V45" s="7" t="n"/>
       <c r="W45" s="7" t="n"/>
       <c r="X45" s="7" t="n"/>
+      <c r="Y45" s="7" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="n"/>
@@ -2702,6 +2787,7 @@
       <c r="V46" s="7" t="n"/>
       <c r="W46" s="7" t="n"/>
       <c r="X46" s="7" t="n"/>
+      <c r="Y46" s="7" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="n"/>
@@ -2728,6 +2814,7 @@
       <c r="V47" s="7" t="n"/>
       <c r="W47" s="7" t="n"/>
       <c r="X47" s="7" t="n"/>
+      <c r="Y47" s="7" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="n"/>
@@ -2754,6 +2841,7 @@
       <c r="V48" s="7" t="n"/>
       <c r="W48" s="7" t="n"/>
       <c r="X48" s="7" t="n"/>
+      <c r="Y48" s="7" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="n"/>
@@ -2780,6 +2868,7 @@
       <c r="V49" s="7" t="n"/>
       <c r="W49" s="7" t="n"/>
       <c r="X49" s="7" t="n"/>
+      <c r="Y49" s="7" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="n"/>
@@ -2806,6 +2895,7 @@
       <c r="V50" s="7" t="n"/>
       <c r="W50" s="7" t="n"/>
       <c r="X50" s="7" t="n"/>
+      <c r="Y50" s="7" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="n"/>
@@ -2832,6 +2922,7 @@
       <c r="V51" s="7" t="n"/>
       <c r="W51" s="7" t="n"/>
       <c r="X51" s="7" t="n"/>
+      <c r="Y51" s="7" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="n"/>
@@ -2858,6 +2949,7 @@
       <c r="V52" s="7" t="n"/>
       <c r="W52" s="7" t="n"/>
       <c r="X52" s="7" t="n"/>
+      <c r="Y52" s="7" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="n"/>
@@ -2884,6 +2976,7 @@
       <c r="V53" s="7" t="n"/>
       <c r="W53" s="7" t="n"/>
       <c r="X53" s="7" t="n"/>
+      <c r="Y53" s="7" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="n"/>
@@ -2910,6 +3003,7 @@
       <c r="V54" s="7" t="n"/>
       <c r="W54" s="7" t="n"/>
       <c r="X54" s="7" t="n"/>
+      <c r="Y54" s="7" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="n"/>
@@ -2936,6 +3030,7 @@
       <c r="V55" s="7" t="n"/>
       <c r="W55" s="7" t="n"/>
       <c r="X55" s="7" t="n"/>
+      <c r="Y55" s="7" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="n"/>
@@ -2962,6 +3057,7 @@
       <c r="V56" s="7" t="n"/>
       <c r="W56" s="7" t="n"/>
       <c r="X56" s="7" t="n"/>
+      <c r="Y56" s="7" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="n"/>
@@ -2988,6 +3084,7 @@
       <c r="V57" s="7" t="n"/>
       <c r="W57" s="7" t="n"/>
       <c r="X57" s="7" t="n"/>
+      <c r="Y57" s="7" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="n"/>
@@ -3014,6 +3111,7 @@
       <c r="V58" s="7" t="n"/>
       <c r="W58" s="7" t="n"/>
       <c r="X58" s="7" t="n"/>
+      <c r="Y58" s="7" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="n"/>
@@ -3040,13 +3138,14 @@
       <c r="V59" s="7" t="n"/>
       <c r="W59" s="7" t="n"/>
       <c r="X59" s="7" t="n"/>
+      <c r="Y59" s="7" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation sqref="R2:R500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Bitte einen Wochentag aus der Liste wählen." prompt="Wochentag wählen (für den Stundenplan)." type="list">
+    <dataValidation sqref="S2:S500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Bitte einen Wochentag aus der Liste wählen." prompt="Wochentag wählen (für den Stundenplan)." type="list">
       <formula1>"Montag,Dienstag,Mittwoch,Donnerstag,Freitag,Samstag,Sonntag"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Deutsch,Englisch,Bilingual"</formula1>
     </dataValidation>
     <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="ECTS als Zahl (0–60)." type="decimal" operator="between">

</xml_diff>